<commit_message>
add reach_score & manipulability_score
</commit_message>
<xml_diff>
--- a/dynamics/src/dynamics/xlsx/task_point.xlsx
+++ b/dynamics/src/dynamics/xlsx/task_point.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -31,6 +31,12 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFd5d5d5"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -64,23 +70,23 @@
   </cellStyleXfs>
   <cellXfs count="7">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
     <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
+      <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
+      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -395,35 +401,35 @@
     <col min="6" max="6" style="6" width="12.43357142857143" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="16.5">
       <c r="A1" s="1">
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="B1" s="1">
-        <v>2</v>
+        <v>0.2</v>
       </c>
       <c r="C1" s="1">
-        <v>3</v>
+        <v>0.1</v>
       </c>
       <c r="D1" s="2">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="E1" s="2">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="F1" s="2">
         <v>0</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
       <c r="A2" s="3">
-        <v>3.980600900199073e-31</v>
+        <v>0.2</v>
       </c>
       <c r="B2" s="3">
-        <v>52.293779505</v>
+        <v>0.1</v>
       </c>
       <c r="C2" s="3">
-        <v>14.91853788</v>
+        <v>0.3</v>
       </c>
       <c r="D2" s="4">
         <v>0</v>
@@ -435,84 +441,84 @@
         <v>0</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="16.5">
       <c r="A3" s="1">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="B3" s="1">
-        <v>5</v>
+        <v>0.3</v>
       </c>
       <c r="C3" s="1">
-        <v>5</v>
+        <v>0.1</v>
       </c>
       <c r="D3" s="2">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="E3" s="2">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F3" s="2">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="16.5">
       <c r="A4" s="1">
-        <v>2</v>
+        <v>0.5</v>
       </c>
       <c r="B4" s="1">
         <v>2</v>
       </c>
       <c r="C4" s="1">
-        <v>2</v>
+        <v>0.5</v>
       </c>
       <c r="D4" s="2">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E4" s="2">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F4" s="2">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="16.5">
       <c r="A5" s="1">
-        <v>2</v>
+        <v>0.4</v>
       </c>
       <c r="B5" s="1">
         <v>3</v>
       </c>
       <c r="C5" s="1">
-        <v>2</v>
+        <v>0.5</v>
       </c>
       <c r="D5" s="2">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E5" s="2">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="F5" s="2">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="16.5">
       <c r="A6" s="1">
-        <v>3</v>
+        <v>0.3</v>
       </c>
       <c r="B6" s="1">
-        <v>5</v>
+        <v>0.8</v>
       </c>
       <c r="C6" s="1">
-        <v>4</v>
+        <v>0.5</v>
       </c>
       <c r="D6" s="2">
-        <v>6</v>
+        <v>0.3</v>
       </c>
       <c r="E6" s="2">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F6" s="2">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add reach & manipulability & fixed reward function
</commit_message>
<xml_diff>
--- a/dynamics/src/dynamics/xlsx/task_point.xlsx
+++ b/dynamics/src/dynamics/xlsx/task_point.xlsx
@@ -446,7 +446,7 @@
         <v>0.1</v>
       </c>
       <c r="B3" s="1">
-        <v>0.3</v>
+        <v>0.1</v>
       </c>
       <c r="C3" s="1">
         <v>0.1</v>
@@ -463,13 +463,13 @@
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="16.5">
       <c r="A4" s="1">
-        <v>0.5</v>
+        <v>0.11</v>
       </c>
       <c r="B4" s="1">
-        <v>2</v>
+        <v>0.2</v>
       </c>
       <c r="C4" s="1">
-        <v>0.5</v>
+        <v>0.1</v>
       </c>
       <c r="D4" s="2">
         <v>0</v>
@@ -483,13 +483,13 @@
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="16.5">
       <c r="A5" s="1">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="B5" s="1">
-        <v>3</v>
+        <v>0.1</v>
       </c>
       <c r="C5" s="1">
-        <v>0.5</v>
+        <v>0.1</v>
       </c>
       <c r="D5" s="2">
         <v>0</v>
@@ -503,13 +503,13 @@
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="16.5">
       <c r="A6" s="1">
-        <v>0.3</v>
+        <v>0.1</v>
       </c>
       <c r="B6" s="1">
-        <v>0.8</v>
+        <v>0.2</v>
       </c>
       <c r="C6" s="1">
-        <v>0.5</v>
+        <v>0.1</v>
       </c>
       <c r="D6" s="2">
         <v>0.3</v>

</xml_diff>